<commit_message>
Small changes in prepared_sentences_m.xlsx
</commit_message>
<xml_diff>
--- a/Sentences/prepared_sentences_m.xlsx
+++ b/Sentences/prepared_sentences_m.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30125"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6BE14D5C-B0B5-478C-B07A-3118A13CE647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7E36D20D-A91B-41FD-BA8B-A09800BB313E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -426,7 +426,7 @@
     <t>Kiedy oni uczą się migać z moim bratem?</t>
   </si>
   <si>
-    <t>ONI, KIEDY, UCZYĆ-SIĘ, MIGAĆ, MÓJ, BRAT</t>
+    <t>ONI, KIEDY, UCZYĆ-SIĘ, MIGAĆ, MÓJ, MĘŻCZYZNA, RODZEŃSTWO</t>
   </si>
   <si>
     <t>Wczoraj rano ty byłeś bardzo zmęczony.</t>

</xml_diff>